<commit_message>
LDO Sweep : 레지스터 Sweep Gap += 2, 100회 측정 후 평균값 사용
</commit_message>
<xml_diff>
--- a/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
+++ b/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XDIC_Common\XD04_A6R1_XD12_A7R1\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869BAE27-5C22-498A-9C2D-6C84A2DF4840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820EA2DD-0E04-4DB0-9CC8-6E36E274E9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
+    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
   </bookViews>
   <sheets>
     <sheet name="fw release" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Number</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -58,10 +58,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>"25. 11. 21</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>이름</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -78,11 +74,31 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>xd04p_iqc_jig_260430.hex</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>LDO Sweep에 대하여 1.65V 이상인 경우 stop</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xd04p_iqc_jig_260403.hex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 03. 31</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 04. 03</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 04. 06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xd04p_iqc_jig_260406.hex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LDO Sweep에 대하여 코드 2step씩 증가, 최소 전압 증가량 1.5mV, 측정간 interval 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -497,7 +513,7 @@
     <col min="2" max="2" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="51.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.58203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
@@ -509,7 +525,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2</v>
@@ -523,7 +539,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>4</v>
@@ -534,13 +550,13 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.45">
@@ -548,17 +564,28 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B6" s="3"/>
+      <c r="B6" s="3">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B7" s="3"/>

</xml_diff>

<commit_message>
LDO Sweep Reg' overflow 문제점 해결
</commit_message>
<xml_diff>
--- a/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
+++ b/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XDIC_Common\XD04_A6R1_XD12_A7R1\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820EA2DD-0E04-4DB0-9CC8-6E36E274E9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE93C18-6F5E-48E9-9A31-F9F85DDFEE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
   </bookViews>
   <sheets>
     <sheet name="fw release" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Number</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -99,6 +99,17 @@
   </si>
   <si>
     <t>LDO Sweep에 대하여 코드 2step씩 증가, 최소 전압 증가량 1.5mV, 측정간 interval 증가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 06. 25</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xd04p_iqc_jig_260625.hex</t>
+  </si>
+  <si>
+    <t>LDO Sweep에 대하여 오버플로우 문제 해결</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -588,7 +599,18 @@
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B7" s="3"/>
+      <c r="B7" s="3">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B8" s="3"/>

</xml_diff>

<commit_message>
serial latency: default, 0x2D번지 : 0x155
</commit_message>
<xml_diff>
--- a/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
+++ b/X-Series/XDIC_Common/XD04_A6R1_XD12_A7R1/Docs/xd04_iqc_jig_fw_release.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XDIC_Common\XD04_A6R1_XD12_A7R1\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE93C18-6F5E-48E9-9A31-F9F85DDFEE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7080DC-41E4-4C56-B657-C41160C08A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
   </bookViews>
@@ -109,7 +109,7 @@
     <t>xd04p_iqc_jig_260625.hex</t>
   </si>
   <si>
-    <t>LDO Sweep에 대하여 오버플로우 문제 해결</t>
+    <t>LDO Sweep에 대하여 오버플로우 문제 해결, initial 시 serial_latency : default, 0x2D번지 : 0x155</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -521,10 +521,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71.83203125" style="1" customWidth="1"/>
     <col min="6" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>

</xml_diff>